<commit_message>
Revised Exception Handling in Pythonn
</commit_message>
<xml_diff>
--- a/Python_Revision_Tracker.xlsx
+++ b/Python_Revision_Tracker.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analytics\Python Programming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{42B3729F-8A20-49D0-B158-38126AA52F1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB0ABF08-1C9C-48A5-A095-53759B9F01DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Python Revision Tracker" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="28">
   <si>
     <t>Python Study &amp; Revision Tracker</t>
   </si>
@@ -82,13 +83,31 @@
     <t>Topic Type</t>
   </si>
   <si>
-    <t>Theory</t>
-  </si>
-  <si>
-    <t>Basic Programs</t>
-  </si>
-  <si>
-    <t>Coding</t>
+    <t>Data Structures in Python</t>
+  </si>
+  <si>
+    <t>Theory + Code</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>Data Science with Python</t>
+  </si>
+  <si>
+    <t>Pandas</t>
+  </si>
+  <si>
+    <t>Numpy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matplotlib </t>
+  </si>
+  <si>
+    <t>Seaborn</t>
+  </si>
+  <si>
+    <t>Advanced Python</t>
   </si>
 </sst>
 </file>
@@ -120,7 +139,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -145,6 +164,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -176,7 +201,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -187,6 +212,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -194,8 +231,8 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -499,7 +536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -510,37 +547,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
+      <c r="A2" s="9"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="4" t="s">
         <v>15</v>
       </c>
     </row>
@@ -581,7 +618,7 @@
         <v>10</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>11</v>
@@ -589,105 +626,184 @@
       <c r="E7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
       <c r="I7" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
-      <c r="B8" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>16</v>
-      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="3"/>
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-    </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
+      <c r="F10" s="6">
+        <f>A12+3</f>
+        <v>46171</v>
+      </c>
+      <c r="G10" s="6">
+        <f>F10+5</f>
+        <v>46176</v>
+      </c>
+      <c r="H10" s="6">
+        <f>G10+15</f>
+        <v>46191</v>
+      </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
+      <c r="A11" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" s="5">
+        <f>DATE(2026,5,26)</f>
+        <v>46168</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
+      <c r="F14" s="6">
+        <f>A16+3</f>
+        <v>46178</v>
+      </c>
+      <c r="G14" s="6">
+        <f>A16+5</f>
+        <v>46180</v>
+      </c>
+      <c r="H14" s="6">
+        <f>A16+15</f>
+        <v>46190</v>
+      </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
+      <c r="A15" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
+      <c r="A16" s="5">
+        <f>DATE(2026,6,2)</f>
+        <v>46175</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>16</v>
+      </c>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
+      <c r="I16" s="2" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
+      <c r="B17" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
@@ -698,7 +814,9 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
+      <c r="B18" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
@@ -709,7 +827,9 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
+      <c r="B19" s="3" t="s">
+        <v>25</v>
+      </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
@@ -720,7 +840,9 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
+      <c r="B20" s="3" t="s">
+        <v>26</v>
+      </c>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
@@ -752,80 +874,135 @@
       <c r="I22" s="3"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
+      <c r="F23" s="6">
+        <f>A25+3</f>
+        <v>3</v>
+      </c>
+      <c r="G23" s="6">
+        <f>F23+5</f>
+        <v>8</v>
+      </c>
+      <c r="H23" s="6">
+        <f>G23+15</f>
+        <v>23</v>
+      </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
-      <c r="I24" s="3"/>
+      <c r="A24" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
+      <c r="A25" s="5"/>
+      <c r="B25" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F25" s="11" t="s">
+        <v>16</v>
+      </c>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
-      <c r="I25" s="3"/>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" s="6" t="s">
+      <c r="I25" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A26" s="3"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A27" s="3"/>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A40" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B28" s="5"/>
-      <c r="C28" s="5"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
-      <c r="F28" s="5"/>
-      <c r="G28" s="5"/>
-      <c r="H28" s="5"/>
-      <c r="I28" s="5"/>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A29" s="5"/>
-      <c r="B29" s="5"/>
-      <c r="C29" s="5"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5"/>
-      <c r="G29" s="5"/>
-      <c r="H29" s="5"/>
-      <c r="I29" s="5"/>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="5"/>
-      <c r="B30" s="5"/>
-      <c r="C30" s="5"/>
-      <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
-      <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
-      <c r="I30" s="5"/>
+      <c r="B40" s="9"/>
+      <c r="C40" s="9"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="9"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="9"/>
+      <c r="I40" s="9"/>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A41" s="9"/>
+      <c r="B41" s="9"/>
+      <c r="C41" s="9"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="9"/>
+      <c r="F41" s="9"/>
+      <c r="G41" s="9"/>
+      <c r="H41" s="9"/>
+      <c r="I41" s="9"/>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A42" s="9"/>
+      <c r="B42" s="9"/>
+      <c r="C42" s="9"/>
+      <c r="D42" s="9"/>
+      <c r="E42" s="9"/>
+      <c r="F42" s="9"/>
+      <c r="G42" s="9"/>
+      <c r="H42" s="9"/>
+      <c r="I42" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:I2"/>
-    <mergeCell ref="A28:I30"/>
+    <mergeCell ref="A40:I42"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F7:H8" xr:uid="{2F8B58AC-D863-4DEC-A42B-25A92B27A5EA}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F7:H8 F12:H12 F16:H16 F25:H25" xr:uid="{2F8B58AC-D863-4DEC-A42B-25A92B27A5EA}">
       <formula1>"Done, Pending"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>